<commit_message>
update with cc_biomass from emmas pkg
</commit_message>
<xml_diff>
--- a/data-raw/clim1/00_keys/treatment-key-v6.xlsx
+++ b/data-raw/clim1/00_keys/treatment-key-v6.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{46CE05BC-E121-4C8E-8B77-D8C04AE5FB05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08D94F36-8B7F-49C7-8831-93BF8F3893FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="field_year_2026" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="71">
   <si>
     <t>trt_nu</t>
   </si>
@@ -42,9 +42,6 @@
     <t>Treatments may change in each establishment year</t>
   </si>
   <si>
-    <t>A perennial legume (Medicago lupulina) planted in its own rows</t>
-  </si>
-  <si>
     <t>An annual legume (Persian clover) planted between the narrow rows, will not grow much in spring and summer, but will grow in the fall</t>
   </si>
   <si>
@@ -115,9 +112,6 @@
   </si>
   <si>
     <t>Rephil perennial rye</t>
-  </si>
-  <si>
-    <t>A tetraploid, would be interesting to include?</t>
   </si>
   <si>
     <t>Perennial wheat from The Land Institute in Kansas USA, may not do very well, but can test it an turn it into a practice plot if it fails</t>
@@ -260,13 +254,16 @@
     <t>p; a</t>
   </si>
   <si>
-    <t>26f_p0leg3</t>
-  </si>
-  <si>
-    <t>p; leg3</t>
-  </si>
-  <si>
-    <t>This is tentative, could be replaced by the Hungarian variety if we get it</t>
+    <t>A tetraploid, would be interesting to include, we have 20 kg seed</t>
+  </si>
+  <si>
+    <t>26f_p0leg2</t>
+  </si>
+  <si>
+    <t>It seems like medicago lupulina should be planted in september</t>
+  </si>
+  <si>
+    <t>A perennial legume (Medicago lupulina) planted in 25 cm spaced rows with perennial rye in between</t>
   </si>
 </sst>
 </file>
@@ -728,126 +725,126 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:L57"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.88671875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.44140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="27.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="13.88671875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="17.88671875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="18.88671875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="32.109375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="63.6640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="27.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="13.85546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.85546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="26.7109375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="63.7109375" style="1" customWidth="1"/>
     <col min="11" max="11" width="34" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="1"/>
+    <col min="12" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>58</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>0</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>33</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>35</v>
       </c>
       <c r="C7" s="6">
         <v>1</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G7" s="6">
         <v>12.5</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I7" s="6">
         <v>300</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K7" s="6"/>
       <c r="L7" s="2"/>
     </row>
-    <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
       <c r="B8" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C8" s="6">
         <v>2</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G8" s="6">
         <v>12.5</v>
@@ -859,29 +856,29 @@
         <v>300</v>
       </c>
       <c r="J8" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="K8" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="K8" s="6" t="s">
-        <v>5</v>
-      </c>
       <c r="L8" s="2"/>
     </row>
-    <row r="9" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
       <c r="B9" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C9" s="6">
         <v>3</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G9" s="6">
         <v>25</v>
@@ -893,95 +890,95 @@
         <v>300</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>3</v>
+        <v>70</v>
       </c>
       <c r="K9" s="6"/>
       <c r="L9" s="2"/>
     </row>
-    <row r="10" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C10" s="6">
         <v>4</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G10" s="6">
         <v>12.5</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I10" s="6">
         <v>300</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K10" s="8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="L10" s="2"/>
     </row>
-    <row r="11" spans="1:12" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
       <c r="B11" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C11" s="6">
         <v>5</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G11" s="6">
         <v>25</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I11" s="6">
         <v>300</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="L11" s="2"/>
     </row>
-    <row r="12" spans="1:12" ht="50.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
       <c r="B12" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C12" s="6">
         <v>6</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G12" s="6">
         <v>12.5</v>
@@ -990,33 +987,33 @@
         <v>80</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K12" s="6"/>
       <c r="L12" s="2"/>
     </row>
-    <row r="13" spans="1:12" ht="58.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="B13" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C13" s="4">
         <v>7</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H13" s="5">
         <v>80</v>
@@ -1025,29 +1022,29 @@
         <v>300</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L13" s="2"/>
     </row>
-    <row r="14" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
       <c r="B14" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C14" s="4">
         <v>8</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G14" s="4">
         <v>12.5</v>
@@ -1059,27 +1056,27 @@
         <v>300</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K14" s="4"/>
       <c r="L14" s="2"/>
     </row>
-    <row r="15" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
       <c r="B15" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C15" s="4">
         <v>9</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G15" s="4">
         <v>12.5</v>
@@ -1091,27 +1088,27 @@
         <v>300</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K15" s="4"/>
       <c r="L15" s="2"/>
     </row>
-    <row r="16" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4"/>
       <c r="B16" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C16" s="4">
         <v>10</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G16" s="4">
         <v>25</v>
@@ -1123,27 +1120,27 @@
         <v>300</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K16" s="4"/>
       <c r="L16" s="2"/>
     </row>
-    <row r="17" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
       <c r="B17" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C17" s="4">
         <v>11</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G17" s="4">
         <v>12.5</v>
@@ -1155,27 +1152,27 @@
         <v>300</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K17" s="4"/>
       <c r="L17" s="2"/>
     </row>
-    <row r="18" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
       <c r="B18" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C18" s="4">
         <v>12</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G18" s="4">
         <v>25</v>
@@ -1187,27 +1184,27 @@
         <v>300</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K18" s="4"/>
       <c r="L18" s="2"/>
     </row>
-    <row r="19" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
       <c r="B19" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C19" s="4">
         <v>13</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G19" s="4">
         <v>25</v>
@@ -1219,27 +1216,27 @@
         <v>300</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K19" s="4"/>
       <c r="L19" s="2"/>
     </row>
-    <row r="20" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
       <c r="B20" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C20" s="4">
         <v>14</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G20" s="4">
         <v>12.5</v>
@@ -1251,27 +1248,27 @@
         <v>300</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K20" s="4"/>
       <c r="L20" s="2"/>
     </row>
-    <row r="21" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4"/>
       <c r="B21" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C21" s="4">
         <v>15</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G21" s="4">
         <v>25</v>
@@ -1283,27 +1280,27 @@
         <v>300</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K21" s="4"/>
       <c r="L21" s="2"/>
     </row>
-    <row r="22" spans="1:12" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5"/>
       <c r="B22" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C22" s="5">
         <v>16</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G22" s="5">
         <v>12.5</v>
@@ -1315,27 +1312,27 @@
         <v>300</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K22" s="5"/>
       <c r="L22" s="2"/>
     </row>
-    <row r="23" spans="1:12" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5"/>
       <c r="B23" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C23" s="5">
         <v>17</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G23" s="5">
         <v>12.5</v>
@@ -1347,27 +1344,27 @@
         <v>300</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="K23" s="5"/>
       <c r="L23" s="2"/>
     </row>
-    <row r="24" spans="1:12" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5"/>
       <c r="B24" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C24" s="5">
         <v>18</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="G24" s="5">
         <v>25</v>
@@ -1379,12 +1376,12 @@
         <v>300</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K24" s="5"/>
       <c r="L24" s="2"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2">
@@ -1400,7 +1397,7 @@
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2">
@@ -1416,7 +1413,7 @@
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2">
@@ -1432,7 +1429,7 @@
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2">
@@ -1448,7 +1445,7 @@
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2">
@@ -1464,7 +1461,7 @@
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2">
@@ -1480,7 +1477,7 @@
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2">
@@ -1496,7 +1493,7 @@
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2">
@@ -1512,7 +1509,7 @@
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2">
@@ -1528,7 +1525,7 @@
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2">
@@ -1544,7 +1541,7 @@
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2">
@@ -1560,7 +1557,7 @@
       <c r="K35" s="2"/>
       <c r="L35" s="2"/>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2">
@@ -1576,7 +1573,7 @@
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2">
@@ -1592,7 +1589,7 @@
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2">
@@ -1608,7 +1605,7 @@
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2">
@@ -1624,7 +1621,7 @@
       <c r="K39" s="2"/>
       <c r="L39" s="2"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2">
@@ -1640,7 +1637,7 @@
       <c r="K40" s="2"/>
       <c r="L40" s="2"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2">
@@ -1656,7 +1653,7 @@
       <c r="K41" s="2"/>
       <c r="L41" s="2"/>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2">
@@ -1672,7 +1669,7 @@
       <c r="K42" s="2"/>
       <c r="L42" s="2"/>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2">
@@ -1688,7 +1685,7 @@
       <c r="K43" s="2"/>
       <c r="L43" s="2"/>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2">
@@ -1704,7 +1701,7 @@
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2">
@@ -1720,7 +1717,7 @@
       <c r="K45" s="2"/>
       <c r="L45" s="2"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2">
@@ -1736,7 +1733,7 @@
       <c r="K46" s="2"/>
       <c r="L46" s="2"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2">
@@ -1752,7 +1749,7 @@
       <c r="K47" s="2"/>
       <c r="L47" s="2"/>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2">
@@ -1768,7 +1765,7 @@
       <c r="K48" s="2"/>
       <c r="L48" s="2"/>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2">
@@ -1784,7 +1781,7 @@
       <c r="K49" s="2"/>
       <c r="L49" s="2"/>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2">
@@ -1800,7 +1797,7 @@
       <c r="K50" s="2"/>
       <c r="L50" s="2"/>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2">
@@ -1816,7 +1813,7 @@
       <c r="K51" s="2"/>
       <c r="L51" s="2"/>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2">
@@ -1832,7 +1829,7 @@
       <c r="K52" s="2"/>
       <c r="L52" s="2"/>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2">
@@ -1848,7 +1845,7 @@
       <c r="K53" s="2"/>
       <c r="L53" s="2"/>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2">
@@ -1864,7 +1861,7 @@
       <c r="K54" s="2"/>
       <c r="L54" s="2"/>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2">
@@ -1880,7 +1877,7 @@
       <c r="K55" s="2"/>
       <c r="L55" s="2"/>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C56" s="2">
         <v>50</v>
       </c>
@@ -1890,7 +1887,7 @@
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C57" s="2">
         <v>51</v>
       </c>
@@ -1908,21 +1905,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"blankspreadsheet","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"blankspreadsheet","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{613AEFFE-C095-42A7-A0AC-5564FFC1D197}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7408D0D6-C97A-426B-8466-DDDAA7A3F420}">
   <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7408D0D6-C97A-426B-8466-DDDAA7A3F420}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{613AEFFE-C095-42A7-A0AC-5564FFC1D197}">
   <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
</xml_diff>